<commit_message>
test: extend sprint 1 security and regression evidence
</commit_message>
<xml_diff>
--- a/docs/testing/sprint-1-test-cases.xlsx
+++ b/docs/testing/sprint-1-test-cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\08_Personals\School Portfolio\GradNavi\docs\testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3FEE0D7-842B-4DDC-ADB2-60A70DECD07A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BAC1651-1062-4440-99F4-90982911F66D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="821" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="849" uniqueCount="427">
   <si>
     <t>GradNavi Sprint 1 Test Dashboard</t>
   </si>
@@ -1254,6 +1254,69 @@
   </si>
   <si>
     <t>Not executable yet because the Student Profile backend API required by this integration test is not available.</t>
+  </si>
+  <si>
+    <t>Django successfully connected to PostgreSQL using the configured backend and gradnavi_db database.</t>
+  </si>
+  <si>
+    <t>EV-020</t>
+  </si>
+  <si>
+    <t>Database connection verified through Django without exposing credentials.</t>
+  </si>
+  <si>
+    <t>Django reported no pending migrations, and showmigrations confirmed all current Sprint 1 migrations are applied.</t>
+  </si>
+  <si>
+    <t>EV-021</t>
+  </si>
+  <si>
+    <t>Migration state verified against the current development database.</t>
+  </si>
+  <si>
+    <t>Protected current-user endpoint rejected a request without JWT authentication and returned 401 Unauthorized without exposing student data.</t>
+  </si>
+  <si>
+    <t>EV-022</t>
+  </si>
+  <si>
+    <t>Verified against /api/v1/auth/me/ without an Authorization header.</t>
+  </si>
+  <si>
+    <t>Invalid authentication returned a controlled 401 error response without exposing traceback information, server file paths, database credentials, SQL statements, secret keys, or internal exception details.</t>
+  </si>
+  <si>
+    <t>EV-023</t>
+  </si>
+  <si>
+    <t>Representative invalid-login request used to verify safe API error handling.</t>
+  </si>
+  <si>
+    <t>No backend secrets, database credentials, or PostgreSQL configuration details were found in the frontend source or production build using the defined secret-pattern searches.</t>
+  </si>
+  <si>
+    <t>EV-016</t>
+  </si>
+  <si>
+    <t>Frontend source and built assets were checked for backend secret/configuration patterns.</t>
+  </si>
+  <si>
+    <t>CORS configuration allows the approved local React origins. The approved localhost origin received Access-Control-Allow-Origin, while the unapproved example.com origin did not.</t>
+  </si>
+  <si>
+    <t>EV-017; EV-018; EV-019</t>
+  </si>
+  <si>
+    <t>Configuration and preflight behaviour verified for approved and unapproved origins.</t>
+  </si>
+  <si>
+    <t>Authentication regression completed successfully after the MainLayout refactor. Protected-route behaviour remained correct after logout, frontend lint completed with 0 warnings and 0 errors, and the production build completed successfully.</t>
+  </si>
+  <si>
+    <t>EV-024; EV-025</t>
+  </si>
+  <si>
+    <t>Regression supported by earlier FE-AUTH evidence for login, session persistence, and logout.</t>
   </si>
 </sst>
 </file>
@@ -1329,8 +1392,9 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1"/>
@@ -1355,18 +1419,19 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="3" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="4" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="3" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{C3C0151A-5983-4143-803C-455A60ADA368}"/>
     <cellStyle name="Normal 3" xfId="2" xr:uid="{3F5EBA85-C488-4D43-98C2-3295708BE0CB}"/>
     <cellStyle name="Normal 4" xfId="3" xr:uid="{B7A6470D-3966-4C63-8A36-BC5385BF686D}"/>
+    <cellStyle name="Normal 5" xfId="4" xr:uid="{D21B6ECE-1049-4548-A94A-F0F14C3CA562}"/>
   </cellStyles>
   <dxfs count="6">
     <dxf>
@@ -1512,7 +1577,7 @@
                   <c:v>61</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>5</c:v>
+                  <c:v>12</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1521,7 +1586,7 @@
                   <c:v>23</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>33</c:v>
+                  <c:v>26</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2011,7 +2076,7 @@
       </c>
       <c r="B5" s="2">
         <f>COUNTIF('Test Cases'!J2:J62,"Pass")</f>
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2" t="s">
@@ -2098,7 +2163,7 @@
       </c>
       <c r="B8" s="2">
         <f>COUNTIF('Test Cases'!J2:J62,"Not Run")</f>
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2" t="s">
@@ -2364,7 +2429,7 @@
       </c>
       <c r="F18" s="2">
         <f>COUNTIFS('Test Cases'!B$2:B$62,D18,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
@@ -2388,7 +2453,7 @@
       </c>
       <c r="F19" s="2">
         <f>COUNTIFS('Test Cases'!B$2:B$62,D19,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G19" s="2"/>
       <c r="H19" s="4" t="s">
@@ -2418,7 +2483,7 @@
       </c>
       <c r="F20" s="2">
         <f>COUNTIFS('Test Cases'!B$2:B$62,D20,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G20" s="2"/>
       <c r="H20" s="2" t="s">
@@ -2454,7 +2519,7 @@
       </c>
       <c r="J21" s="2">
         <f>COUNTIFS('Test Cases'!P$2:P$62,H21,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
@@ -2478,7 +2543,7 @@
       </c>
       <c r="J22" s="2">
         <f>COUNTIFS('Test Cases'!P$2:P$62,H22,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
@@ -2502,7 +2567,7 @@
       </c>
       <c r="J23" s="2">
         <f>COUNTIFS('Test Cases'!P$2:P$62,H23,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
@@ -4699,7 +4764,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="53" spans="1:16" ht="29.25">
+    <row r="53" spans="1:16" ht="57.75">
       <c r="A53" s="2" t="s">
         <v>294</v>
       </c>
@@ -4724,20 +4789,30 @@
       <c r="H53" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="I53" s="7"/>
+      <c r="I53" s="7" t="s">
+        <v>406</v>
+      </c>
       <c r="J53" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="K53" s="7"/>
-      <c r="L53" s="8"/>
-      <c r="M53" s="7"/>
+        <v>8</v>
+      </c>
+      <c r="K53" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L53" s="8">
+        <v>46256</v>
+      </c>
+      <c r="M53" s="7" t="s">
+        <v>407</v>
+      </c>
       <c r="N53" s="7"/>
-      <c r="O53" s="7"/>
+      <c r="O53" s="7" t="s">
+        <v>408</v>
+      </c>
       <c r="P53" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="54" spans="1:16">
+    <row r="54" spans="1:16" ht="57">
       <c r="A54" s="2" t="s">
         <v>299</v>
       </c>
@@ -4762,15 +4837,25 @@
       <c r="H54" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="I54" s="7"/>
+      <c r="I54" s="7" t="s">
+        <v>409</v>
+      </c>
       <c r="J54" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="K54" s="7"/>
-      <c r="L54" s="8"/>
-      <c r="M54" s="7"/>
+        <v>8</v>
+      </c>
+      <c r="K54" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L54" s="8">
+        <v>46256</v>
+      </c>
+      <c r="M54" s="7" t="s">
+        <v>410</v>
+      </c>
       <c r="N54" s="7"/>
-      <c r="O54" s="7"/>
+      <c r="O54" s="7" t="s">
+        <v>411</v>
+      </c>
       <c r="P54" s="2" t="s">
         <v>36</v>
       </c>
@@ -4813,7 +4898,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="56" spans="1:16" ht="29.25">
+    <row r="56" spans="1:16" ht="72">
       <c r="A56" s="2" t="s">
         <v>309</v>
       </c>
@@ -4838,20 +4923,30 @@
       <c r="H56" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="I56" s="7"/>
+      <c r="I56" s="7" t="s">
+        <v>412</v>
+      </c>
       <c r="J56" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="K56" s="7"/>
-      <c r="L56" s="8"/>
-      <c r="M56" s="7"/>
+        <v>8</v>
+      </c>
+      <c r="K56" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L56" s="8">
+        <v>46256</v>
+      </c>
+      <c r="M56" s="7" t="s">
+        <v>413</v>
+      </c>
       <c r="N56" s="7"/>
-      <c r="O56" s="7"/>
+      <c r="O56" s="7" t="s">
+        <v>414</v>
+      </c>
       <c r="P56" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="57" spans="1:16" ht="29.25">
+    <row r="57" spans="1:16" ht="100.5">
       <c r="A57" s="2" t="s">
         <v>314</v>
       </c>
@@ -4876,20 +4971,30 @@
       <c r="H57" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="I57" s="7"/>
+      <c r="I57" s="7" t="s">
+        <v>415</v>
+      </c>
       <c r="J57" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="K57" s="7"/>
-      <c r="L57" s="8"/>
-      <c r="M57" s="7"/>
+        <v>8</v>
+      </c>
+      <c r="K57" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L57" s="8">
+        <v>46256</v>
+      </c>
+      <c r="M57" s="7" t="s">
+        <v>416</v>
+      </c>
       <c r="N57" s="7"/>
-      <c r="O57" s="7"/>
+      <c r="O57" s="7" t="s">
+        <v>417</v>
+      </c>
       <c r="P57" s="2" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="58" spans="1:16" ht="28.5">
+    <row r="58" spans="1:16" ht="85.5">
       <c r="A58" s="2" t="s">
         <v>319</v>
       </c>
@@ -4914,20 +5019,30 @@
       <c r="H58" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="I58" s="7"/>
+      <c r="I58" s="7" t="s">
+        <v>418</v>
+      </c>
       <c r="J58" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="K58" s="7"/>
-      <c r="L58" s="8"/>
-      <c r="M58" s="7"/>
+        <v>8</v>
+      </c>
+      <c r="K58" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L58" s="8">
+        <v>46256</v>
+      </c>
+      <c r="M58" s="7" t="s">
+        <v>419</v>
+      </c>
       <c r="N58" s="7"/>
-      <c r="O58" s="7"/>
+      <c r="O58" s="7" t="s">
+        <v>420</v>
+      </c>
       <c r="P58" s="2" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="59" spans="1:16">
+    <row r="59" spans="1:16" ht="85.5">
       <c r="A59" s="2" t="s">
         <v>324</v>
       </c>
@@ -4952,20 +5067,30 @@
       <c r="H59" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="I59" s="7"/>
+      <c r="I59" s="7" t="s">
+        <v>421</v>
+      </c>
       <c r="J59" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="K59" s="7"/>
-      <c r="L59" s="8"/>
-      <c r="M59" s="7"/>
+        <v>8</v>
+      </c>
+      <c r="K59" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L59" s="8">
+        <v>46256</v>
+      </c>
+      <c r="M59" s="7" t="s">
+        <v>422</v>
+      </c>
       <c r="N59" s="7"/>
-      <c r="O59" s="7"/>
+      <c r="O59" s="7" t="s">
+        <v>423</v>
+      </c>
       <c r="P59" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="60" spans="1:16" ht="29.25">
+    <row r="60" spans="1:16" ht="114.75">
       <c r="A60" s="2" t="s">
         <v>329</v>
       </c>
@@ -4990,15 +5115,25 @@
       <c r="H60" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="I60" s="7"/>
+      <c r="I60" s="7" t="s">
+        <v>424</v>
+      </c>
       <c r="J60" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="K60" s="7"/>
-      <c r="L60" s="8"/>
-      <c r="M60" s="7"/>
+        <v>8</v>
+      </c>
+      <c r="K60" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L60" s="8">
+        <v>46256</v>
+      </c>
+      <c r="M60" s="7" t="s">
+        <v>425</v>
+      </c>
       <c r="N60" s="7"/>
-      <c r="O60" s="7"/>
+      <c r="O60" s="7" t="s">
+        <v>426</v>
+      </c>
       <c r="P60" s="2" t="s">
         <v>37</v>
       </c>

</xml_diff>

<commit_message>
test: add WBS 4.8 profile integration evidence
</commit_message>
<xml_diff>
--- a/docs/testing/sprint-1-test-cases.xlsx
+++ b/docs/testing/sprint-1-test-cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\08_Personals\School Portfolio\GradNavi\docs\testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BAC1651-1062-4440-99F4-90982911F66D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A69C2A0E-351C-43A0-B4E2-F4080431556A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="849" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="464">
   <si>
     <t>GradNavi Sprint 1 Test Dashboard</t>
   </si>
@@ -1202,9 +1202,6 @@
     <t>Person who actually executes the test and records the result</t>
   </si>
   <si>
-    <t>Waiting for MD's Student Profile backend implementation. No backend profile result is claimed.</t>
-  </si>
-  <si>
     <t>EV-001; EV-002; EV-003; EV-004; EV-005; EV-006</t>
   </si>
   <si>
@@ -1232,12 +1229,6 @@
     <t>Frontend logout behaviour verified.</t>
   </si>
   <si>
-    <t>Waiting for MD's Student Profile backend implementation. Frontend UI exists, but backend data load/update/persistence cannot be verified yet.</t>
-  </si>
-  <si>
-    <t>Not executable yet because the Student Profile backend/API implementation required by this test is pending.</t>
-  </si>
-  <si>
     <t>Registration through React succeeded. Valid registration returned 201; weak-password and duplicate-email errors were displayed; password mismatch was blocked by frontend validation.</t>
   </si>
   <si>
@@ -1253,9 +1244,6 @@
     <t>Logout returned the frontend to /login and cleared GradNavi access token, refresh token, and stored-user entries from localStorage.</t>
   </si>
   <si>
-    <t>Not executable yet because the Student Profile backend API required by this integration test is not available.</t>
-  </si>
-  <si>
     <t>Django successfully connected to PostgreSQL using the configured backend and gradnavi_db database.</t>
   </si>
   <si>
@@ -1317,6 +1305,129 @@
   </si>
   <si>
     <t>Regression supported by earlier FE-AUTH evidence for login, session persistence, and logout.</t>
+  </si>
+  <si>
+    <t>Authenticated WBS 4.8 test student opened /profile. GET /api/v1/profile/ returned HTTP 200 and the student's profile loaded in React.</t>
+  </si>
+  <si>
+    <t>2026-08-28</t>
+  </si>
+  <si>
+    <t>EV-027; EV-028</t>
+  </si>
+  <si>
+    <t>Own-profile retrieval verified through the user-scoped endpoint. Cross-student isolation remains a separate ownership test.</t>
+  </si>
+  <si>
+    <t>GET /api/v1/profile/ returned HTTP 200 and persisted profile sections were displayed through the Student Profile UI across the reload, edit, and deletion checks.</t>
+  </si>
+  <si>
+    <t>EV-028; EV-029; EV-030</t>
+  </si>
+  <si>
+    <t>WBS 4.8 browser evidence confirms the implemented profile collections are returned and rendered. Raw JSON schema inspection remains separate.</t>
+  </si>
+  <si>
+    <t>An existing Education record was edited, Save Profile submitted PATCH successfully, the updated description persisted, and unrelated profile sections remained present after refresh.</t>
+  </si>
+  <si>
+    <t>EV-029</t>
+  </si>
+  <si>
+    <t>Valid authenticated profile update verified through the integrated React and Django flow.</t>
+  </si>
+  <si>
+    <t>Profile changes persisted after successful PATCH requests and browser refreshes. Edited Education remained updated and the removed Project did not return.</t>
+  </si>
+  <si>
+    <t>EV-026; EV-028; EV-029; EV-030</t>
+  </si>
+  <si>
+    <t>Persistence verified through save-and-reload behaviour. Direct database inspection is not claimed by this evidence package.</t>
+  </si>
+  <si>
+    <t>WBS 4.6 backend and WBS 4.8 integration are available. This test remains pending execution.</t>
+  </si>
+  <si>
+    <t>Python with Proficient proficiency was added through the Student Profile UI, saved, and remained visible after browser refresh.</t>
+  </si>
+  <si>
+    <t>EV-028</t>
+  </si>
+  <si>
+    <t>Sprint 1 used prepared shared Skill reference records. Formal reference-data API remains under later work.</t>
+  </si>
+  <si>
+    <t>Artificial Intelligence was selected from the prepared shared Interest references, saved, and remained visible after browser refresh.</t>
+  </si>
+  <si>
+    <t>Interest category remained shared reference data and was not edited by the student.</t>
+  </si>
+  <si>
+    <t>A CQUniversity Master of Information Technology Education record was present in the saved profile and its description remained updated after Save Profile and refresh.</t>
+  </si>
+  <si>
+    <t>Education persistence and edit behaviour verified through the UI.</t>
+  </si>
+  <si>
+    <t>A Software Developer Experience record remained visible in the Student Profile during the refresh and edit verification flow.</t>
+  </si>
+  <si>
+    <t>Experience persistence is visible in the same refreshed profile used for the Education edit check.</t>
+  </si>
+  <si>
+    <t>The available WBS 4.8 screenshots do not prove the current-role date validation result.</t>
+  </si>
+  <si>
+    <t>A project record was part of the WBS 4.8 profile flow and was later removed successfully. The deletion remained persisted after Save Profile and refresh.</t>
+  </si>
+  <si>
+    <t>EV-030</t>
+  </si>
+  <si>
+    <t>EV-030 proves the saved deletion state. A dedicated pre-deletion project screenshot was not captured.</t>
+  </si>
+  <si>
+    <t>The available WBS 4.8 screenshots do not clearly prove a persisted Career Goal record.</t>
+  </si>
+  <si>
+    <t>The available WBS 4.8 screenshots show the questionnaire and save state but do not clearly prove stored response values.</t>
+  </si>
+  <si>
+    <t>2026-08-22</t>
+  </si>
+  <si>
+    <t>Authenticated Student Profile page loaded successfully. GET /api/v1/profile/ returned HTTP 200 and saved Student Profile data displayed after refresh.</t>
+  </si>
+  <si>
+    <t>Frontend GET integration verified.</t>
+  </si>
+  <si>
+    <t>Student added, edited and removed profile data, then used the single Save Profile action. PATCH /api/v1/profile/ returned HTTP 200 and the UI displayed a successful save state.</t>
+  </si>
+  <si>
+    <t>EV-026; EV-027; EV-029; EV-030</t>
+  </si>
+  <si>
+    <t>Frontend PATCH integration verified across add, edit and remove flows.</t>
+  </si>
+  <si>
+    <t>Saved profile information remained after browser refresh. Edited Education remained updated and the removed Project did not return.</t>
+  </si>
+  <si>
+    <t>Reload persistence verified.</t>
+  </si>
+  <si>
+    <t>The five WBS 4.8 screenshots prove UI persistence but do not constitute direct database relationship inspection.</t>
+  </si>
+  <si>
+    <t>Core Sprint 1 happy-path flow passed through registration, login, current-user retrieval, profile GET, profile PATCH, refresh persistence, and the previously verified logout behaviour.</t>
+  </si>
+  <si>
+    <t>EV-014; EV-027; EV-028; EV-030</t>
+  </si>
+  <si>
+    <t>Core happy-path regression passed. Remaining negative/validation cases stay tracked separately.</t>
   </si>
 </sst>
 </file>
@@ -1348,7 +1459,7 @@
       <name val="Carlito"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1375,6 +1486,16 @@
         <fgColor rgb="FFD9EAF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF7FBFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAF4EA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1392,14 +1513,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="5">
+  <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1419,21 +1542,38 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="4" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="6"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="6" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="6" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="6" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="6" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="6" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="5">
+  <cellStyles count="7">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{C3C0151A-5983-4143-803C-455A60ADA368}"/>
     <cellStyle name="Normal 3" xfId="2" xr:uid="{3F5EBA85-C488-4D43-98C2-3295708BE0CB}"/>
     <cellStyle name="Normal 4" xfId="3" xr:uid="{B7A6470D-3966-4C63-8A36-BC5385BF686D}"/>
     <cellStyle name="Normal 5" xfId="4" xr:uid="{D21B6ECE-1049-4548-A94A-F0F14C3CA562}"/>
+    <cellStyle name="Normal 6" xfId="5" xr:uid="{A272D506-DD9B-45F8-B6DB-6ECC05A3878B}"/>
+    <cellStyle name="Normal 7" xfId="6" xr:uid="{79E18355-8E1B-40C8-A0B1-8C02409F04F1}"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="9">
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF666666"/>
@@ -1577,16 +1717,16 @@
                   <c:v>61</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>12</c:v>
+                  <c:v>25</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>23</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>26</c:v>
+                  <c:v>36</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1735,13 +1875,13 @@
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Preconditions"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Test Steps"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Expected Result"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Actual Result"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Actual Result" dataDxfId="1"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Status"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Tester"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Test Date"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Evidence ID"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Evidence ID" dataDxfId="2"/>
     <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Defect Reference"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Notes"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Notes" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2076,7 +2216,7 @@
       </c>
       <c r="B5" s="2">
         <f>COUNTIF('Test Cases'!J2:J62,"Pass")</f>
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2" t="s">
@@ -2134,7 +2274,7 @@
       </c>
       <c r="B7" s="2">
         <f>COUNTIF('Test Cases'!J2:J62,"Blocked")</f>
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2" t="s">
@@ -2146,7 +2286,7 @@
       </c>
       <c r="F7" s="2">
         <f>COUNTIFS('Test Cases'!B$2:B$62,D7,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
@@ -2163,7 +2303,7 @@
       </c>
       <c r="B8" s="2">
         <f>COUNTIF('Test Cases'!J2:J62,"Not Run")</f>
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2" t="s">
@@ -2199,7 +2339,7 @@
       </c>
       <c r="F9" s="2">
         <f>COUNTIFS('Test Cases'!B$2:B$62,D9,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
@@ -2223,7 +2363,7 @@
       </c>
       <c r="F10" s="2">
         <f>COUNTIFS('Test Cases'!B$2:B$62,D10,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
@@ -2251,7 +2391,7 @@
       </c>
       <c r="F11" s="2">
         <f>COUNTIFS('Test Cases'!B$2:B$62,D11,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
@@ -2268,7 +2408,7 @@
       </c>
       <c r="B12" s="2" t="str">
         <f>IF(COUNTIFS('Test Cases'!D2:D62,"Critical",'Test Cases'!J2:J62,"Fail")+COUNTIFS('Test Cases'!D2:D62,"Critical",'Test Cases'!J2:J62,"Blocked")&gt;0,"NOT READY",IF(COUNTIFS('Test Cases'!D2:D62,"Critical",'Test Cases'!J2:J62,"Not Run")&gt;0,"PENDING","READY"))</f>
-        <v>NOT READY</v>
+        <v>PENDING</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2" t="s">
@@ -2280,7 +2420,7 @@
       </c>
       <c r="F12" s="2">
         <f>COUNTIFS('Test Cases'!B$2:B$62,D12,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
@@ -2297,7 +2437,7 @@
       </c>
       <c r="B13" s="2" t="str">
         <f>IF(COUNTIFS('Test Cases'!C2:C62,"Integration",'Test Cases'!J2:J62,"Fail")+COUNTIFS('Test Cases'!C2:C62,"Integration",'Test Cases'!J2:J62,"Blocked")&gt;0,"NOT READY",IF(COUNTIFS('Test Cases'!C2:C62,"Integration",'Test Cases'!J2:J62,"Not Run")&gt;0,"PENDING","READY"))</f>
-        <v>NOT READY</v>
+        <v>PENDING</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2" t="s">
@@ -2309,7 +2449,7 @@
       </c>
       <c r="F13" s="2">
         <f>COUNTIFS('Test Cases'!B$2:B$62,D13,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
@@ -2405,7 +2545,7 @@
       </c>
       <c r="F17" s="2">
         <f>COUNTIFS('Test Cases'!B$2:B$62,D17,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
@@ -2483,7 +2623,7 @@
       </c>
       <c r="F20" s="2">
         <f>COUNTIFS('Test Cases'!B$2:B$62,D20,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G20" s="2"/>
       <c r="H20" s="2" t="s">
@@ -2495,7 +2635,7 @@
       </c>
       <c r="J20" s="2">
         <f>COUNTIFS('Test Cases'!P$2:P$62,H20,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K20" s="2"/>
       <c r="L20" s="2"/>
@@ -2519,7 +2659,7 @@
       </c>
       <c r="J21" s="2">
         <f>COUNTIFS('Test Cases'!P$2:P$62,H21,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="K21" s="2"/>
       <c r="L21" s="2"/>
@@ -2543,7 +2683,7 @@
       </c>
       <c r="J22" s="2">
         <f>COUNTIFS('Test Cases'!P$2:P$62,H22,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="K22" s="2"/>
       <c r="L22" s="2"/>
@@ -2567,7 +2707,7 @@
       </c>
       <c r="J23" s="2">
         <f>COUNTIFS('Test Cases'!P$2:P$62,H23,'Test Cases'!J$2:J$62,"Pass")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K23" s="2"/>
       <c r="L23" s="2"/>
@@ -2630,7 +2770,7 @@
     <col min="10" max="10" width="12" customWidth="1"/>
     <col min="11" max="11" width="16" customWidth="1"/>
     <col min="12" max="12" width="13" customWidth="1"/>
-    <col min="13" max="13" width="14" customWidth="1"/>
+    <col min="13" max="13" width="14" style="2" customWidth="1"/>
     <col min="14" max="14" width="18" customWidth="1"/>
     <col min="15" max="15" width="24" customWidth="1"/>
     <col min="16" max="16" width="14" customWidth="1"/>
@@ -2711,16 +2851,16 @@
       <c r="H2" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="I2" s="7"/>
+      <c r="I2" s="10"/>
       <c r="J2" s="7" t="s">
         <v>14</v>
       </c>
       <c r="K2" s="7"/>
-      <c r="L2" s="8"/>
-      <c r="M2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="10"/>
       <c r="N2" s="7"/>
-      <c r="O2" s="7"/>
-      <c r="P2" s="2" t="s">
+      <c r="O2" s="10"/>
+      <c r="P2" s="7" t="s">
         <v>34</v>
       </c>
     </row>
@@ -2749,16 +2889,16 @@
       <c r="H3" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="I3" s="7"/>
+      <c r="I3" s="10"/>
       <c r="J3" s="7" t="s">
         <v>14</v>
       </c>
       <c r="K3" s="7"/>
-      <c r="L3" s="8"/>
-      <c r="M3" s="7"/>
+      <c r="L3" s="7"/>
+      <c r="M3" s="10"/>
       <c r="N3" s="7"/>
-      <c r="O3" s="7"/>
-      <c r="P3" s="2" t="s">
+      <c r="O3" s="10"/>
+      <c r="P3" s="7" t="s">
         <v>34</v>
       </c>
     </row>
@@ -2787,16 +2927,16 @@
       <c r="H4" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="I4" s="7"/>
+      <c r="I4" s="10"/>
       <c r="J4" s="7" t="s">
         <v>14</v>
       </c>
       <c r="K4" s="7"/>
-      <c r="L4" s="8"/>
-      <c r="M4" s="7"/>
+      <c r="L4" s="7"/>
+      <c r="M4" s="10"/>
       <c r="N4" s="7"/>
-      <c r="O4" s="7"/>
-      <c r="P4" s="2" t="s">
+      <c r="O4" s="10"/>
+      <c r="P4" s="7" t="s">
         <v>34</v>
       </c>
     </row>
@@ -2825,16 +2965,16 @@
       <c r="H5" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="I5" s="7"/>
+      <c r="I5" s="10"/>
       <c r="J5" s="7" t="s">
         <v>14</v>
       </c>
       <c r="K5" s="7"/>
-      <c r="L5" s="8"/>
-      <c r="M5" s="7"/>
+      <c r="L5" s="7"/>
+      <c r="M5" s="10"/>
       <c r="N5" s="7"/>
-      <c r="O5" s="7"/>
-      <c r="P5" s="2" t="s">
+      <c r="O5" s="10"/>
+      <c r="P5" s="7" t="s">
         <v>34</v>
       </c>
     </row>
@@ -2863,16 +3003,16 @@
       <c r="H6" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="I6" s="7"/>
+      <c r="I6" s="10"/>
       <c r="J6" s="7" t="s">
         <v>14</v>
       </c>
       <c r="K6" s="7"/>
-      <c r="L6" s="8"/>
-      <c r="M6" s="7"/>
+      <c r="L6" s="7"/>
+      <c r="M6" s="10"/>
       <c r="N6" s="7"/>
-      <c r="O6" s="7"/>
-      <c r="P6" s="2" t="s">
+      <c r="O6" s="10"/>
+      <c r="P6" s="7" t="s">
         <v>34</v>
       </c>
     </row>
@@ -2901,16 +3041,16 @@
       <c r="H7" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="I7" s="7"/>
+      <c r="I7" s="10"/>
       <c r="J7" s="7" t="s">
         <v>14</v>
       </c>
       <c r="K7" s="7"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="7"/>
+      <c r="L7" s="7"/>
+      <c r="M7" s="10"/>
       <c r="N7" s="7"/>
-      <c r="O7" s="7"/>
-      <c r="P7" s="2" t="s">
+      <c r="O7" s="10"/>
+      <c r="P7" s="7" t="s">
         <v>34</v>
       </c>
     </row>
@@ -2939,16 +3079,16 @@
       <c r="H8" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I8" s="7"/>
+      <c r="I8" s="10"/>
       <c r="J8" s="7" t="s">
         <v>14</v>
       </c>
       <c r="K8" s="7"/>
-      <c r="L8" s="8"/>
-      <c r="M8" s="7"/>
+      <c r="L8" s="7"/>
+      <c r="M8" s="10"/>
       <c r="N8" s="7"/>
-      <c r="O8" s="7"/>
-      <c r="P8" s="2" t="s">
+      <c r="O8" s="10"/>
+      <c r="P8" s="7" t="s">
         <v>34</v>
       </c>
     </row>
@@ -2977,16 +3117,16 @@
       <c r="H9" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="I9" s="7"/>
+      <c r="I9" s="10"/>
       <c r="J9" s="7" t="s">
         <v>14</v>
       </c>
       <c r="K9" s="7"/>
-      <c r="L9" s="8"/>
-      <c r="M9" s="7"/>
+      <c r="L9" s="7"/>
+      <c r="M9" s="10"/>
       <c r="N9" s="7"/>
-      <c r="O9" s="7"/>
-      <c r="P9" s="2" t="s">
+      <c r="O9" s="10"/>
+      <c r="P9" s="7" t="s">
         <v>34</v>
       </c>
     </row>
@@ -3015,16 +3155,16 @@
       <c r="H10" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="I10" s="7"/>
+      <c r="I10" s="10"/>
       <c r="J10" s="7" t="s">
         <v>14</v>
       </c>
       <c r="K10" s="7"/>
-      <c r="L10" s="8"/>
-      <c r="M10" s="7"/>
+      <c r="L10" s="7"/>
+      <c r="M10" s="10"/>
       <c r="N10" s="7"/>
-      <c r="O10" s="7"/>
-      <c r="P10" s="2" t="s">
+      <c r="O10" s="10"/>
+      <c r="P10" s="7" t="s">
         <v>34</v>
       </c>
     </row>
@@ -3053,16 +3193,16 @@
       <c r="H11" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="I11" s="7"/>
+      <c r="I11" s="10"/>
       <c r="J11" s="7" t="s">
         <v>14</v>
       </c>
       <c r="K11" s="7"/>
-      <c r="L11" s="8"/>
-      <c r="M11" s="7"/>
+      <c r="L11" s="7"/>
+      <c r="M11" s="10"/>
       <c r="N11" s="7"/>
-      <c r="O11" s="7"/>
-      <c r="P11" s="2" t="s">
+      <c r="O11" s="10"/>
+      <c r="P11" s="7" t="s">
         <v>34</v>
       </c>
     </row>
@@ -3091,16 +3231,16 @@
       <c r="H12" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="I12" s="7"/>
+      <c r="I12" s="10"/>
       <c r="J12" s="7" t="s">
         <v>14</v>
       </c>
       <c r="K12" s="7"/>
-      <c r="L12" s="8"/>
-      <c r="M12" s="7"/>
+      <c r="L12" s="7"/>
+      <c r="M12" s="10"/>
       <c r="N12" s="7"/>
-      <c r="O12" s="7"/>
-      <c r="P12" s="2" t="s">
+      <c r="O12" s="10"/>
+      <c r="P12" s="7" t="s">
         <v>34</v>
       </c>
     </row>
@@ -3129,16 +3269,16 @@
       <c r="H13" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="I13" s="7"/>
+      <c r="I13" s="10"/>
       <c r="J13" s="7" t="s">
         <v>14</v>
       </c>
       <c r="K13" s="7"/>
-      <c r="L13" s="8"/>
-      <c r="M13" s="7"/>
+      <c r="L13" s="7"/>
+      <c r="M13" s="10"/>
       <c r="N13" s="7"/>
-      <c r="O13" s="7"/>
-      <c r="P13" s="2" t="s">
+      <c r="O13" s="10"/>
+      <c r="P13" s="7" t="s">
         <v>34</v>
       </c>
     </row>
@@ -3167,16 +3307,16 @@
       <c r="H14" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="I14" s="7"/>
+      <c r="I14" s="10"/>
       <c r="J14" s="7" t="s">
         <v>14</v>
       </c>
       <c r="K14" s="7"/>
-      <c r="L14" s="8"/>
-      <c r="M14" s="7"/>
+      <c r="L14" s="7"/>
+      <c r="M14" s="10"/>
       <c r="N14" s="7"/>
-      <c r="O14" s="7"/>
-      <c r="P14" s="2" t="s">
+      <c r="O14" s="10"/>
+      <c r="P14" s="7" t="s">
         <v>34</v>
       </c>
     </row>
@@ -3205,16 +3345,16 @@
       <c r="H15" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="I15" s="7"/>
+      <c r="I15" s="10"/>
       <c r="J15" s="7" t="s">
         <v>14</v>
       </c>
       <c r="K15" s="7"/>
-      <c r="L15" s="8"/>
-      <c r="M15" s="7"/>
+      <c r="L15" s="7"/>
+      <c r="M15" s="10"/>
       <c r="N15" s="7"/>
-      <c r="O15" s="7"/>
-      <c r="P15" s="2" t="s">
+      <c r="O15" s="10"/>
+      <c r="P15" s="7" t="s">
         <v>34</v>
       </c>
     </row>
@@ -3243,20 +3383,20 @@
       <c r="H16" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="I16" s="7"/>
+      <c r="I16" s="10"/>
       <c r="J16" s="7" t="s">
         <v>14</v>
       </c>
       <c r="K16" s="7"/>
-      <c r="L16" s="8"/>
-      <c r="M16" s="7"/>
+      <c r="L16" s="7"/>
+      <c r="M16" s="10"/>
       <c r="N16" s="7"/>
-      <c r="O16" s="7"/>
-      <c r="P16" s="2" t="s">
+      <c r="O16" s="10"/>
+      <c r="P16" s="7" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="17" spans="1:16" ht="29.25">
+    <row r="17" spans="1:16" ht="72">
       <c r="A17" s="2" t="s">
         <v>129</v>
       </c>
@@ -3281,16 +3421,26 @@
       <c r="H17" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="I17" s="7"/>
-      <c r="J17" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="K17" s="7"/>
-      <c r="L17" s="8"/>
-      <c r="M17" s="7"/>
-      <c r="N17" s="7"/>
-      <c r="O17" s="7"/>
-      <c r="P17" s="2" t="s">
+      <c r="I17" s="11" t="s">
+        <v>423</v>
+      </c>
+      <c r="J17" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="K17" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="L17" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="M17" s="11" t="s">
+        <v>425</v>
+      </c>
+      <c r="N17" s="8"/>
+      <c r="O17" s="11" t="s">
+        <v>426</v>
+      </c>
+      <c r="P17" s="8" t="s">
         <v>34</v>
       </c>
     </row>
@@ -3319,20 +3469,20 @@
       <c r="H18" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="I18" s="7"/>
-      <c r="J18" s="7" t="s">
+      <c r="I18" s="11"/>
+      <c r="J18" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="K18" s="7"/>
+      <c r="K18" s="8"/>
       <c r="L18" s="8"/>
-      <c r="M18" s="7"/>
-      <c r="N18" s="7"/>
-      <c r="O18" s="7"/>
-      <c r="P18" s="2" t="s">
+      <c r="M18" s="11"/>
+      <c r="N18" s="8"/>
+      <c r="O18" s="11"/>
+      <c r="P18" s="8" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="1:16" ht="28.5">
+    <row r="19" spans="1:16" ht="85.5">
       <c r="A19" s="2" t="s">
         <v>138</v>
       </c>
@@ -3357,20 +3507,30 @@
       <c r="H19" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="I19" s="7"/>
-      <c r="J19" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="K19" s="7"/>
-      <c r="L19" s="8"/>
-      <c r="M19" s="7"/>
-      <c r="N19" s="7"/>
-      <c r="O19" s="7"/>
-      <c r="P19" s="2" t="s">
+      <c r="I19" s="11" t="s">
+        <v>427</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="K19" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="L19" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="M19" s="11" t="s">
+        <v>428</v>
+      </c>
+      <c r="N19" s="8"/>
+      <c r="O19" s="11" t="s">
+        <v>429</v>
+      </c>
+      <c r="P19" s="8" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="1:16" ht="29.25">
+    <row r="20" spans="1:16" ht="100.5">
       <c r="A20" s="2" t="s">
         <v>143</v>
       </c>
@@ -3395,16 +3555,26 @@
       <c r="H20" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="I20" s="7"/>
-      <c r="J20" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="K20" s="7"/>
-      <c r="L20" s="8"/>
-      <c r="M20" s="7"/>
-      <c r="N20" s="7"/>
-      <c r="O20" s="7"/>
-      <c r="P20" s="2" t="s">
+      <c r="I20" s="11" t="s">
+        <v>430</v>
+      </c>
+      <c r="J20" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="K20" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="L20" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="M20" s="11" t="s">
+        <v>431</v>
+      </c>
+      <c r="N20" s="8"/>
+      <c r="O20" s="11" t="s">
+        <v>432</v>
+      </c>
+      <c r="P20" s="8" t="s">
         <v>34</v>
       </c>
     </row>
@@ -3433,16 +3603,16 @@
       <c r="H21" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="I21" s="7"/>
-      <c r="J21" s="7" t="s">
+      <c r="I21" s="11"/>
+      <c r="J21" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="K21" s="7"/>
+      <c r="K21" s="8"/>
       <c r="L21" s="8"/>
-      <c r="M21" s="7"/>
-      <c r="N21" s="7"/>
-      <c r="O21" s="7"/>
-      <c r="P21" s="2" t="s">
+      <c r="M21" s="11"/>
+      <c r="N21" s="8"/>
+      <c r="O21" s="11"/>
+      <c r="P21" s="8" t="s">
         <v>34</v>
       </c>
     </row>
@@ -3471,16 +3641,16 @@
       <c r="H22" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="I22" s="7"/>
-      <c r="J22" s="7" t="s">
+      <c r="I22" s="11"/>
+      <c r="J22" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="K22" s="7"/>
+      <c r="K22" s="8"/>
       <c r="L22" s="8"/>
-      <c r="M22" s="7"/>
-      <c r="N22" s="7"/>
-      <c r="O22" s="7"/>
-      <c r="P22" s="2" t="s">
+      <c r="M22" s="11"/>
+      <c r="N22" s="8"/>
+      <c r="O22" s="11"/>
+      <c r="P22" s="8" t="s">
         <v>34</v>
       </c>
     </row>
@@ -3509,20 +3679,20 @@
       <c r="H23" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="I23" s="7"/>
-      <c r="J23" s="7" t="s">
+      <c r="I23" s="11"/>
+      <c r="J23" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="K23" s="7"/>
+      <c r="K23" s="8"/>
       <c r="L23" s="8"/>
-      <c r="M23" s="7"/>
-      <c r="N23" s="7"/>
-      <c r="O23" s="7"/>
-      <c r="P23" s="2" t="s">
+      <c r="M23" s="11"/>
+      <c r="N23" s="8"/>
+      <c r="O23" s="11"/>
+      <c r="P23" s="8" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="24" spans="1:16">
+    <row r="24" spans="1:16" ht="85.5">
       <c r="A24" s="2" t="s">
         <v>160</v>
       </c>
@@ -3547,20 +3717,30 @@
       <c r="H24" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="I24" s="7"/>
-      <c r="J24" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="K24" s="7"/>
-      <c r="L24" s="8"/>
-      <c r="M24" s="7"/>
-      <c r="N24" s="7"/>
-      <c r="O24" s="7"/>
-      <c r="P24" s="2" t="s">
+      <c r="I24" s="12" t="s">
+        <v>433</v>
+      </c>
+      <c r="J24" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="K24" s="9" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="25" spans="1:16" ht="72">
+      <c r="L24" s="9" t="s">
+        <v>424</v>
+      </c>
+      <c r="M24" s="12" t="s">
+        <v>434</v>
+      </c>
+      <c r="N24" s="9"/>
+      <c r="O24" s="12" t="s">
+        <v>435</v>
+      </c>
+      <c r="P24" s="9" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" ht="57.75">
       <c r="A25" s="2" t="s">
         <v>164</v>
       </c>
@@ -3585,24 +3765,22 @@
       <c r="H25" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="I25" s="7" t="s">
-        <v>399</v>
-      </c>
+      <c r="I25" s="10"/>
       <c r="J25" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K25" s="7"/>
-      <c r="L25" s="8"/>
-      <c r="M25" s="7"/>
+      <c r="L25" s="7"/>
+      <c r="M25" s="10"/>
       <c r="N25" s="7"/>
-      <c r="O25" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="P25" s="2" t="s">
+      <c r="O25" s="10" t="s">
+        <v>436</v>
+      </c>
+      <c r="P25" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="72">
+    <row r="26" spans="1:16" ht="57.75">
       <c r="A26" s="2" t="s">
         <v>170</v>
       </c>
@@ -3627,24 +3805,22 @@
       <c r="H26" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="I26" s="7" t="s">
-        <v>399</v>
-      </c>
+      <c r="I26" s="10"/>
       <c r="J26" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K26" s="7"/>
-      <c r="L26" s="8"/>
-      <c r="M26" s="7"/>
+      <c r="L26" s="7"/>
+      <c r="M26" s="10"/>
       <c r="N26" s="7"/>
-      <c r="O26" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="P26" s="2" t="s">
+      <c r="O26" s="10" t="s">
+        <v>436</v>
+      </c>
+      <c r="P26" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="27" spans="1:16" ht="72">
+    <row r="27" spans="1:16" ht="57.75">
       <c r="A27" s="2" t="s">
         <v>173</v>
       </c>
@@ -3669,24 +3845,22 @@
       <c r="H27" s="2" t="s">
         <v>176</v>
       </c>
-      <c r="I27" s="7" t="s">
-        <v>399</v>
-      </c>
+      <c r="I27" s="10"/>
       <c r="J27" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K27" s="7"/>
-      <c r="L27" s="8"/>
-      <c r="M27" s="7"/>
+      <c r="L27" s="7"/>
+      <c r="M27" s="10"/>
       <c r="N27" s="7"/>
-      <c r="O27" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="P27" s="2" t="s">
+      <c r="O27" s="10" t="s">
+        <v>436</v>
+      </c>
+      <c r="P27" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="28" spans="1:16" ht="72">
+    <row r="28" spans="1:16" ht="57.75">
       <c r="A28" s="2" t="s">
         <v>177</v>
       </c>
@@ -3711,20 +3885,18 @@
       <c r="H28" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="I28" s="7" t="s">
-        <v>399</v>
-      </c>
+      <c r="I28" s="10"/>
       <c r="J28" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K28" s="7"/>
-      <c r="L28" s="8"/>
-      <c r="M28" s="7"/>
+      <c r="L28" s="7"/>
+      <c r="M28" s="10"/>
       <c r="N28" s="7"/>
-      <c r="O28" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="P28" s="2" t="s">
+      <c r="O28" s="10" t="s">
+        <v>436</v>
+      </c>
+      <c r="P28" s="7" t="s">
         <v>36</v>
       </c>
     </row>
@@ -3753,24 +3925,30 @@
       <c r="H29" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="I29" s="7" t="s">
-        <v>399</v>
+      <c r="I29" s="10" t="s">
+        <v>437</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="K29" s="7"/>
-      <c r="L29" s="8"/>
-      <c r="M29" s="7"/>
+        <v>8</v>
+      </c>
+      <c r="K29" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L29" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="M29" s="10" t="s">
+        <v>438</v>
+      </c>
       <c r="N29" s="7"/>
-      <c r="O29" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="P29" s="2" t="s">
+      <c r="O29" s="10" t="s">
+        <v>439</v>
+      </c>
+      <c r="P29" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="30" spans="1:16" ht="71.25">
+    <row r="30" spans="1:16" ht="57">
       <c r="A30" s="2" t="s">
         <v>186</v>
       </c>
@@ -3795,24 +3973,22 @@
       <c r="H30" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="I30" s="7" t="s">
-        <v>399</v>
-      </c>
+      <c r="I30" s="10"/>
       <c r="J30" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K30" s="7"/>
-      <c r="L30" s="8"/>
-      <c r="M30" s="7"/>
+      <c r="L30" s="7"/>
+      <c r="M30" s="10"/>
       <c r="N30" s="7"/>
-      <c r="O30" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="P30" s="2" t="s">
+      <c r="O30" s="10" t="s">
+        <v>436</v>
+      </c>
+      <c r="P30" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="31" spans="1:16" ht="71.25">
+    <row r="31" spans="1:16" ht="57">
       <c r="A31" s="2" t="s">
         <v>191</v>
       </c>
@@ -3837,24 +4013,22 @@
       <c r="H31" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="I31" s="7" t="s">
-        <v>399</v>
-      </c>
+      <c r="I31" s="10"/>
       <c r="J31" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K31" s="7"/>
-      <c r="L31" s="8"/>
-      <c r="M31" s="7"/>
+      <c r="L31" s="7"/>
+      <c r="M31" s="10"/>
       <c r="N31" s="7"/>
-      <c r="O31" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="P31" s="2" t="s">
+      <c r="O31" s="10" t="s">
+        <v>436</v>
+      </c>
+      <c r="P31" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="32" spans="1:16" ht="71.25">
+    <row r="32" spans="1:16" ht="57">
       <c r="A32" s="2" t="s">
         <v>197</v>
       </c>
@@ -3879,20 +4053,18 @@
       <c r="H32" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="I32" s="7" t="s">
-        <v>399</v>
-      </c>
+      <c r="I32" s="10"/>
       <c r="J32" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K32" s="7"/>
-      <c r="L32" s="8"/>
-      <c r="M32" s="7"/>
+      <c r="L32" s="7"/>
+      <c r="M32" s="10"/>
       <c r="N32" s="7"/>
-      <c r="O32" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="P32" s="2" t="s">
+      <c r="O32" s="10" t="s">
+        <v>436</v>
+      </c>
+      <c r="P32" s="7" t="s">
         <v>36</v>
       </c>
     </row>
@@ -3921,24 +4093,30 @@
       <c r="H33" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="I33" s="7" t="s">
-        <v>399</v>
+      <c r="I33" s="10" t="s">
+        <v>440</v>
       </c>
       <c r="J33" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="K33" s="7"/>
-      <c r="L33" s="8"/>
-      <c r="M33" s="7"/>
+        <v>8</v>
+      </c>
+      <c r="K33" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L33" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="M33" s="10" t="s">
+        <v>438</v>
+      </c>
       <c r="N33" s="7"/>
-      <c r="O33" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="P33" s="2" t="s">
+      <c r="O33" s="10" t="s">
+        <v>441</v>
+      </c>
+      <c r="P33" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="34" spans="1:16" ht="71.25">
+    <row r="34" spans="1:16" ht="57">
       <c r="A34" s="2" t="s">
         <v>206</v>
       </c>
@@ -3963,24 +4141,22 @@
       <c r="H34" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="I34" s="7" t="s">
-        <v>399</v>
-      </c>
+      <c r="I34" s="10"/>
       <c r="J34" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K34" s="7"/>
-      <c r="L34" s="8"/>
-      <c r="M34" s="7"/>
+      <c r="L34" s="7"/>
+      <c r="M34" s="10"/>
       <c r="N34" s="7"/>
-      <c r="O34" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="P34" s="2" t="s">
+      <c r="O34" s="10" t="s">
+        <v>436</v>
+      </c>
+      <c r="P34" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="35" spans="1:16" ht="71.25">
+    <row r="35" spans="1:16" ht="57">
       <c r="A35" s="2" t="s">
         <v>209</v>
       </c>
@@ -4005,24 +4181,22 @@
       <c r="H35" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="I35" s="7" t="s">
-        <v>399</v>
-      </c>
+      <c r="I35" s="10"/>
       <c r="J35" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K35" s="7"/>
-      <c r="L35" s="8"/>
-      <c r="M35" s="7"/>
+      <c r="L35" s="7"/>
+      <c r="M35" s="10"/>
       <c r="N35" s="7"/>
-      <c r="O35" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="P35" s="2" t="s">
+      <c r="O35" s="10" t="s">
+        <v>436</v>
+      </c>
+      <c r="P35" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="36" spans="1:16" ht="71.25">
+    <row r="36" spans="1:16" ht="85.5">
       <c r="A36" s="2" t="s">
         <v>214</v>
       </c>
@@ -4047,24 +4221,30 @@
       <c r="H36" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="I36" s="7" t="s">
-        <v>399</v>
+      <c r="I36" s="10" t="s">
+        <v>442</v>
       </c>
       <c r="J36" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="K36" s="7"/>
-      <c r="L36" s="8"/>
-      <c r="M36" s="7"/>
+        <v>8</v>
+      </c>
+      <c r="K36" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L36" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="M36" s="10" t="s">
+        <v>431</v>
+      </c>
       <c r="N36" s="7"/>
-      <c r="O36" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="P36" s="2" t="s">
+      <c r="O36" s="10" t="s">
+        <v>443</v>
+      </c>
+      <c r="P36" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="37" spans="1:16" ht="71.25">
+    <row r="37" spans="1:16" ht="57">
       <c r="A37" s="2" t="s">
         <v>219</v>
       </c>
@@ -4089,20 +4269,18 @@
       <c r="H37" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="I37" s="7" t="s">
-        <v>399</v>
-      </c>
+      <c r="I37" s="10"/>
       <c r="J37" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K37" s="7"/>
-      <c r="L37" s="8"/>
-      <c r="M37" s="7"/>
+      <c r="L37" s="7"/>
+      <c r="M37" s="10"/>
       <c r="N37" s="7"/>
-      <c r="O37" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="P37" s="2" t="s">
+      <c r="O37" s="10" t="s">
+        <v>436</v>
+      </c>
+      <c r="P37" s="7" t="s">
         <v>36</v>
       </c>
     </row>
@@ -4131,24 +4309,30 @@
       <c r="H38" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="I38" s="7" t="s">
-        <v>399</v>
+      <c r="I38" s="10" t="s">
+        <v>444</v>
       </c>
       <c r="J38" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="K38" s="7"/>
-      <c r="L38" s="8"/>
-      <c r="M38" s="7"/>
+        <v>8</v>
+      </c>
+      <c r="K38" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L38" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="M38" s="10" t="s">
+        <v>431</v>
+      </c>
       <c r="N38" s="7"/>
-      <c r="O38" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="P38" s="2" t="s">
+      <c r="O38" s="10" t="s">
+        <v>445</v>
+      </c>
+      <c r="P38" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="39" spans="1:16" ht="71.25">
+    <row r="39" spans="1:16" ht="57">
       <c r="A39" s="2" t="s">
         <v>227</v>
       </c>
@@ -4173,20 +4357,18 @@
       <c r="H39" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="I39" s="7" t="s">
-        <v>399</v>
-      </c>
+      <c r="I39" s="10"/>
       <c r="J39" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K39" s="7"/>
-      <c r="L39" s="8"/>
-      <c r="M39" s="7"/>
+      <c r="L39" s="7"/>
+      <c r="M39" s="10"/>
       <c r="N39" s="7"/>
-      <c r="O39" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="P39" s="2" t="s">
+      <c r="O39" s="10" t="s">
+        <v>446</v>
+      </c>
+      <c r="P39" s="7" t="s">
         <v>36</v>
       </c>
     </row>
@@ -4215,24 +4397,30 @@
       <c r="H40" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="I40" s="7" t="s">
-        <v>399</v>
+      <c r="I40" s="10" t="s">
+        <v>447</v>
       </c>
       <c r="J40" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="K40" s="7"/>
-      <c r="L40" s="8"/>
-      <c r="M40" s="7"/>
+        <v>8</v>
+      </c>
+      <c r="K40" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L40" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="M40" s="10" t="s">
+        <v>448</v>
+      </c>
       <c r="N40" s="7"/>
-      <c r="O40" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="P40" s="2" t="s">
+      <c r="O40" s="10" t="s">
+        <v>449</v>
+      </c>
+      <c r="P40" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="41" spans="1:16" ht="71.25">
+    <row r="41" spans="1:16" ht="57">
       <c r="A41" s="2" t="s">
         <v>235</v>
       </c>
@@ -4257,24 +4445,22 @@
       <c r="H41" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="I41" s="7" t="s">
-        <v>399</v>
-      </c>
+      <c r="I41" s="10"/>
       <c r="J41" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K41" s="7"/>
-      <c r="L41" s="8"/>
-      <c r="M41" s="7"/>
+      <c r="L41" s="7"/>
+      <c r="M41" s="10"/>
       <c r="N41" s="7"/>
-      <c r="O41" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="P41" s="2" t="s">
+      <c r="O41" s="10" t="s">
+        <v>436</v>
+      </c>
+      <c r="P41" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="42" spans="1:16" ht="71.25">
+    <row r="42" spans="1:16" ht="57">
       <c r="A42" s="2" t="s">
         <v>240</v>
       </c>
@@ -4299,24 +4485,22 @@
       <c r="H42" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="I42" s="7" t="s">
-        <v>399</v>
-      </c>
+      <c r="I42" s="10"/>
       <c r="J42" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K42" s="7"/>
-      <c r="L42" s="8"/>
-      <c r="M42" s="7"/>
+      <c r="L42" s="7"/>
+      <c r="M42" s="10"/>
       <c r="N42" s="7"/>
-      <c r="O42" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="P42" s="2" t="s">
+      <c r="O42" s="10" t="s">
+        <v>450</v>
+      </c>
+      <c r="P42" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="43" spans="1:16" ht="71.25">
+    <row r="43" spans="1:16" ht="85.5">
       <c r="A43" s="2" t="s">
         <v>244</v>
       </c>
@@ -4341,20 +4525,18 @@
       <c r="H43" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="I43" s="7" t="s">
-        <v>399</v>
-      </c>
+      <c r="I43" s="10"/>
       <c r="J43" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K43" s="7"/>
-      <c r="L43" s="8"/>
-      <c r="M43" s="7"/>
+      <c r="L43" s="7"/>
+      <c r="M43" s="10"/>
       <c r="N43" s="7"/>
-      <c r="O43" s="7" t="s">
-        <v>388</v>
-      </c>
-      <c r="P43" s="2" t="s">
+      <c r="O43" s="10" t="s">
+        <v>451</v>
+      </c>
+      <c r="P43" s="7" t="s">
         <v>36</v>
       </c>
     </row>
@@ -4383,8 +4565,8 @@
       <c r="H44" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="I44" s="7" t="s">
-        <v>400</v>
+      <c r="I44" s="10" t="s">
+        <v>397</v>
       </c>
       <c r="J44" s="7" t="s">
         <v>8</v>
@@ -4392,17 +4574,17 @@
       <c r="K44" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="L44" s="8">
-        <v>46256</v>
-      </c>
-      <c r="M44" s="7" t="s">
+      <c r="L44" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="M44" s="10" t="s">
+        <v>388</v>
+      </c>
+      <c r="N44" s="7"/>
+      <c r="O44" s="10" t="s">
         <v>389</v>
       </c>
-      <c r="N44" s="7"/>
-      <c r="O44" s="7" t="s">
-        <v>390</v>
-      </c>
-      <c r="P44" s="2" t="s">
+      <c r="P44" s="7" t="s">
         <v>35</v>
       </c>
     </row>
@@ -4431,8 +4613,8 @@
       <c r="H45" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="I45" s="7" t="s">
-        <v>401</v>
+      <c r="I45" s="10" t="s">
+        <v>398</v>
       </c>
       <c r="J45" s="7" t="s">
         <v>8</v>
@@ -4440,17 +4622,17 @@
       <c r="K45" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="L45" s="8">
-        <v>46256</v>
-      </c>
-      <c r="M45" s="7" t="s">
+      <c r="L45" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="M45" s="10" t="s">
+        <v>390</v>
+      </c>
+      <c r="N45" s="7"/>
+      <c r="O45" s="10" t="s">
         <v>391</v>
       </c>
-      <c r="N45" s="7"/>
-      <c r="O45" s="7" t="s">
-        <v>392</v>
-      </c>
-      <c r="P45" s="2" t="s">
+      <c r="P45" s="7" t="s">
         <v>35</v>
       </c>
     </row>
@@ -4479,8 +4661,8 @@
       <c r="H46" s="2" t="s">
         <v>263</v>
       </c>
-      <c r="I46" s="7" t="s">
-        <v>402</v>
+      <c r="I46" s="10" t="s">
+        <v>399</v>
       </c>
       <c r="J46" s="7" t="s">
         <v>8</v>
@@ -4488,17 +4670,17 @@
       <c r="K46" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="L46" s="8">
-        <v>46256</v>
-      </c>
-      <c r="M46" s="7" t="s">
+      <c r="L46" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="M46" s="10" t="s">
+        <v>392</v>
+      </c>
+      <c r="N46" s="7"/>
+      <c r="O46" s="10" t="s">
         <v>393</v>
       </c>
-      <c r="N46" s="7"/>
-      <c r="O46" s="7" t="s">
-        <v>394</v>
-      </c>
-      <c r="P46" s="2" t="s">
+      <c r="P46" s="7" t="s">
         <v>35</v>
       </c>
     </row>
@@ -4527,8 +4709,8 @@
       <c r="H47" s="2" t="s">
         <v>268</v>
       </c>
-      <c r="I47" s="7" t="s">
-        <v>403</v>
+      <c r="I47" s="10" t="s">
+        <v>400</v>
       </c>
       <c r="J47" s="7" t="s">
         <v>8</v>
@@ -4536,15 +4718,15 @@
       <c r="K47" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="L47" s="8">
-        <v>46256</v>
-      </c>
-      <c r="M47" s="7"/>
+      <c r="L47" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="M47" s="10"/>
       <c r="N47" s="7"/>
-      <c r="O47" s="7" t="s">
-        <v>395</v>
-      </c>
-      <c r="P47" s="2" t="s">
+      <c r="O47" s="10" t="s">
+        <v>394</v>
+      </c>
+      <c r="P47" s="7" t="s">
         <v>35</v>
       </c>
     </row>
@@ -4573,8 +4755,8 @@
       <c r="H48" s="2" t="s">
         <v>273</v>
       </c>
-      <c r="I48" s="7" t="s">
-        <v>404</v>
+      <c r="I48" s="10" t="s">
+        <v>401</v>
       </c>
       <c r="J48" s="7" t="s">
         <v>8</v>
@@ -4582,21 +4764,21 @@
       <c r="K48" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="L48" s="8">
-        <v>46256</v>
-      </c>
-      <c r="M48" s="7" t="s">
+      <c r="L48" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="M48" s="10" t="s">
+        <v>395</v>
+      </c>
+      <c r="N48" s="7"/>
+      <c r="O48" s="10" t="s">
         <v>396</v>
       </c>
-      <c r="N48" s="7"/>
-      <c r="O48" s="7" t="s">
-        <v>397</v>
-      </c>
-      <c r="P48" s="2" t="s">
+      <c r="P48" s="7" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="49" spans="1:16" ht="86.25">
+    <row r="49" spans="1:16" ht="72">
       <c r="A49" s="2" t="s">
         <v>274</v>
       </c>
@@ -4621,20 +4803,26 @@
       <c r="H49" s="2" t="s">
         <v>278</v>
       </c>
-      <c r="I49" s="7" t="s">
-        <v>405</v>
-      </c>
-      <c r="J49" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="K49" s="7"/>
-      <c r="L49" s="8"/>
-      <c r="M49" s="7"/>
-      <c r="N49" s="7"/>
-      <c r="O49" s="7" t="s">
-        <v>398</v>
-      </c>
-      <c r="P49" s="2" t="s">
+      <c r="I49" s="11" t="s">
+        <v>453</v>
+      </c>
+      <c r="J49" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="K49" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="L49" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="M49" s="11" t="s">
+        <v>438</v>
+      </c>
+      <c r="N49" s="8"/>
+      <c r="O49" s="11" t="s">
+        <v>454</v>
+      </c>
+      <c r="P49" s="8" t="s">
         <v>35</v>
       </c>
     </row>
@@ -4663,24 +4851,30 @@
       <c r="H50" s="2" t="s">
         <v>283</v>
       </c>
-      <c r="I50" s="7" t="s">
-        <v>405</v>
-      </c>
-      <c r="J50" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="K50" s="7"/>
-      <c r="L50" s="8"/>
-      <c r="M50" s="7"/>
-      <c r="N50" s="7"/>
-      <c r="O50" s="7" t="s">
-        <v>398</v>
-      </c>
-      <c r="P50" s="2" t="s">
+      <c r="I50" s="11" t="s">
+        <v>455</v>
+      </c>
+      <c r="J50" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="K50" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="L50" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="M50" s="11" t="s">
+        <v>456</v>
+      </c>
+      <c r="N50" s="8"/>
+      <c r="O50" s="11" t="s">
+        <v>457</v>
+      </c>
+      <c r="P50" s="8" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="51" spans="1:16" ht="85.5">
+    <row r="51" spans="1:16" ht="57">
       <c r="A51" s="2" t="s">
         <v>284</v>
       </c>
@@ -4705,24 +4899,22 @@
       <c r="H51" s="2" t="s">
         <v>288</v>
       </c>
-      <c r="I51" s="7" t="s">
-        <v>405</v>
-      </c>
-      <c r="J51" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="K51" s="7"/>
+      <c r="I51" s="11"/>
+      <c r="J51" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="K51" s="8"/>
       <c r="L51" s="8"/>
-      <c r="M51" s="7"/>
-      <c r="N51" s="7"/>
-      <c r="O51" s="7" t="s">
-        <v>398</v>
-      </c>
-      <c r="P51" s="2" t="s">
+      <c r="M51" s="11"/>
+      <c r="N51" s="8"/>
+      <c r="O51" s="11" t="s">
+        <v>436</v>
+      </c>
+      <c r="P51" s="8" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="52" spans="1:16" ht="85.5">
+    <row r="52" spans="1:16" ht="71.25">
       <c r="A52" s="2" t="s">
         <v>289</v>
       </c>
@@ -4747,20 +4939,26 @@
       <c r="H52" s="2" t="s">
         <v>293</v>
       </c>
-      <c r="I52" s="7" t="s">
-        <v>405</v>
-      </c>
-      <c r="J52" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="K52" s="7"/>
-      <c r="L52" s="8"/>
-      <c r="M52" s="7"/>
-      <c r="N52" s="7"/>
-      <c r="O52" s="7" t="s">
-        <v>398</v>
-      </c>
-      <c r="P52" s="2" t="s">
+      <c r="I52" s="11" t="s">
+        <v>458</v>
+      </c>
+      <c r="J52" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="K52" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="L52" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="M52" s="11" t="s">
+        <v>428</v>
+      </c>
+      <c r="N52" s="8"/>
+      <c r="O52" s="11" t="s">
+        <v>459</v>
+      </c>
+      <c r="P52" s="8" t="s">
         <v>35</v>
       </c>
     </row>
@@ -4789,8 +4987,8 @@
       <c r="H53" s="2" t="s">
         <v>298</v>
       </c>
-      <c r="I53" s="7" t="s">
-        <v>406</v>
+      <c r="I53" s="10" t="s">
+        <v>402</v>
       </c>
       <c r="J53" s="7" t="s">
         <v>8</v>
@@ -4798,17 +4996,17 @@
       <c r="K53" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="L53" s="8">
-        <v>46256</v>
-      </c>
-      <c r="M53" s="7" t="s">
-        <v>407</v>
+      <c r="L53" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="M53" s="10" t="s">
+        <v>403</v>
       </c>
       <c r="N53" s="7"/>
-      <c r="O53" s="7" t="s">
-        <v>408</v>
-      </c>
-      <c r="P53" s="2" t="s">
+      <c r="O53" s="10" t="s">
+        <v>404</v>
+      </c>
+      <c r="P53" s="7" t="s">
         <v>36</v>
       </c>
     </row>
@@ -4837,8 +5035,8 @@
       <c r="H54" s="2" t="s">
         <v>303</v>
       </c>
-      <c r="I54" s="7" t="s">
-        <v>409</v>
+      <c r="I54" s="10" t="s">
+        <v>405</v>
       </c>
       <c r="J54" s="7" t="s">
         <v>8</v>
@@ -4846,21 +5044,21 @@
       <c r="K54" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="L54" s="8">
-        <v>46256</v>
-      </c>
-      <c r="M54" s="7" t="s">
-        <v>410</v>
+      <c r="L54" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="M54" s="10" t="s">
+        <v>406</v>
       </c>
       <c r="N54" s="7"/>
-      <c r="O54" s="7" t="s">
-        <v>411</v>
-      </c>
-      <c r="P54" s="2" t="s">
+      <c r="O54" s="10" t="s">
+        <v>407</v>
+      </c>
+      <c r="P54" s="7" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="55" spans="1:16" ht="28.5">
+    <row r="55" spans="1:16" ht="71.25">
       <c r="A55" s="2" t="s">
         <v>304</v>
       </c>
@@ -4885,16 +5083,18 @@
       <c r="H55" s="2" t="s">
         <v>308</v>
       </c>
-      <c r="I55" s="7"/>
+      <c r="I55" s="10"/>
       <c r="J55" s="7" t="s">
         <v>14</v>
       </c>
       <c r="K55" s="7"/>
-      <c r="L55" s="8"/>
-      <c r="M55" s="7"/>
+      <c r="L55" s="7"/>
+      <c r="M55" s="10"/>
       <c r="N55" s="7"/>
-      <c r="O55" s="7"/>
-      <c r="P55" s="2" t="s">
+      <c r="O55" s="10" t="s">
+        <v>460</v>
+      </c>
+      <c r="P55" s="7" t="s">
         <v>37</v>
       </c>
     </row>
@@ -4923,8 +5123,8 @@
       <c r="H56" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="I56" s="7" t="s">
-        <v>412</v>
+      <c r="I56" s="10" t="s">
+        <v>408</v>
       </c>
       <c r="J56" s="7" t="s">
         <v>8</v>
@@ -4932,17 +5132,17 @@
       <c r="K56" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="L56" s="8">
-        <v>46256</v>
-      </c>
-      <c r="M56" s="7" t="s">
-        <v>413</v>
+      <c r="L56" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="M56" s="10" t="s">
+        <v>409</v>
       </c>
       <c r="N56" s="7"/>
-      <c r="O56" s="7" t="s">
-        <v>414</v>
-      </c>
-      <c r="P56" s="2" t="s">
+      <c r="O56" s="10" t="s">
+        <v>410</v>
+      </c>
+      <c r="P56" s="7" t="s">
         <v>37</v>
       </c>
     </row>
@@ -4971,8 +5171,8 @@
       <c r="H57" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="I57" s="7" t="s">
-        <v>415</v>
+      <c r="I57" s="10" t="s">
+        <v>411</v>
       </c>
       <c r="J57" s="7" t="s">
         <v>8</v>
@@ -4980,17 +5180,17 @@
       <c r="K57" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="L57" s="8">
-        <v>46256</v>
-      </c>
-      <c r="M57" s="7" t="s">
-        <v>416</v>
+      <c r="L57" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="M57" s="10" t="s">
+        <v>412</v>
       </c>
       <c r="N57" s="7"/>
-      <c r="O57" s="7" t="s">
-        <v>417</v>
-      </c>
-      <c r="P57" s="2" t="s">
+      <c r="O57" s="10" t="s">
+        <v>413</v>
+      </c>
+      <c r="P57" s="7" t="s">
         <v>37</v>
       </c>
     </row>
@@ -5019,8 +5219,8 @@
       <c r="H58" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="I58" s="7" t="s">
-        <v>418</v>
+      <c r="I58" s="10" t="s">
+        <v>414</v>
       </c>
       <c r="J58" s="7" t="s">
         <v>8</v>
@@ -5028,17 +5228,17 @@
       <c r="K58" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="L58" s="8">
-        <v>46256</v>
-      </c>
-      <c r="M58" s="7" t="s">
-        <v>419</v>
+      <c r="L58" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="M58" s="10" t="s">
+        <v>415</v>
       </c>
       <c r="N58" s="7"/>
-      <c r="O58" s="7" t="s">
-        <v>420</v>
-      </c>
-      <c r="P58" s="2" t="s">
+      <c r="O58" s="10" t="s">
+        <v>416</v>
+      </c>
+      <c r="P58" s="7" t="s">
         <v>35</v>
       </c>
     </row>
@@ -5067,8 +5267,8 @@
       <c r="H59" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="I59" s="7" t="s">
-        <v>421</v>
+      <c r="I59" s="10" t="s">
+        <v>417</v>
       </c>
       <c r="J59" s="7" t="s">
         <v>8</v>
@@ -5076,17 +5276,17 @@
       <c r="K59" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="L59" s="8">
-        <v>46256</v>
-      </c>
-      <c r="M59" s="7" t="s">
-        <v>422</v>
+      <c r="L59" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="M59" s="10" t="s">
+        <v>418</v>
       </c>
       <c r="N59" s="7"/>
-      <c r="O59" s="7" t="s">
-        <v>423</v>
-      </c>
-      <c r="P59" s="2" t="s">
+      <c r="O59" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="P59" s="7" t="s">
         <v>36</v>
       </c>
     </row>
@@ -5115,8 +5315,8 @@
       <c r="H60" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="I60" s="7" t="s">
-        <v>424</v>
+      <c r="I60" s="10" t="s">
+        <v>420</v>
       </c>
       <c r="J60" s="7" t="s">
         <v>8</v>
@@ -5124,17 +5324,17 @@
       <c r="K60" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="L60" s="8">
-        <v>46256</v>
-      </c>
-      <c r="M60" s="7" t="s">
-        <v>425</v>
+      <c r="L60" s="7" t="s">
+        <v>452</v>
+      </c>
+      <c r="M60" s="10" t="s">
+        <v>421</v>
       </c>
       <c r="N60" s="7"/>
-      <c r="O60" s="7" t="s">
-        <v>426</v>
-      </c>
-      <c r="P60" s="2" t="s">
+      <c r="O60" s="10" t="s">
+        <v>422</v>
+      </c>
+      <c r="P60" s="7" t="s">
         <v>37</v>
       </c>
     </row>
@@ -5163,20 +5363,20 @@
       <c r="H61" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="I61" s="7"/>
+      <c r="I61" s="10"/>
       <c r="J61" s="7" t="s">
         <v>14</v>
       </c>
       <c r="K61" s="7"/>
-      <c r="L61" s="8"/>
-      <c r="M61" s="7"/>
+      <c r="L61" s="7"/>
+      <c r="M61" s="10"/>
       <c r="N61" s="7"/>
-      <c r="O61" s="7"/>
-      <c r="P61" s="2" t="s">
+      <c r="O61" s="10"/>
+      <c r="P61" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="62" spans="1:16" ht="28.5">
+    <row r="62" spans="1:16" ht="99.75">
       <c r="A62" s="2" t="s">
         <v>339</v>
       </c>
@@ -5201,39 +5401,49 @@
       <c r="H62" s="2" t="s">
         <v>343</v>
       </c>
-      <c r="I62" s="7"/>
+      <c r="I62" s="10" t="s">
+        <v>461</v>
+      </c>
       <c r="J62" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="K62" s="7"/>
-      <c r="L62" s="8"/>
-      <c r="M62" s="7"/>
+        <v>8</v>
+      </c>
+      <c r="K62" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L62" s="7" t="s">
+        <v>424</v>
+      </c>
+      <c r="M62" s="10" t="s">
+        <v>462</v>
+      </c>
       <c r="N62" s="7"/>
-      <c r="O62" s="7"/>
-      <c r="P62" s="2" t="s">
+      <c r="O62" s="10" t="s">
+        <v>463</v>
+      </c>
+      <c r="P62" s="7" t="s">
         <v>37</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="D2:D62">
-    <cfRule type="expression" dxfId="5" priority="5">
+    <cfRule type="expression" dxfId="8" priority="5">
       <formula>D2="Critical"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="6">
+    <cfRule type="expression" dxfId="7" priority="6">
       <formula>D2="High"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2:J62">
-    <cfRule type="expression" dxfId="3" priority="1">
+    <cfRule type="expression" dxfId="6" priority="1">
       <formula>J2="Pass"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="2">
+    <cfRule type="expression" dxfId="5" priority="2">
       <formula>J2="Fail"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="1" priority="3">
+    <cfRule type="expression" dxfId="4" priority="3">
       <formula>J2="Blocked"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="4">
+    <cfRule type="expression" dxfId="3" priority="4">
       <formula>J2="Not Run"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>